<commit_message>
feat(BarridoOne): :sparkles: Genera el mensaje por whats y envia la foto
</commit_message>
<xml_diff>
--- a/assets/Informe_Tiempos_Actualizados.xlsx
+++ b/assets/Informe_Tiempos_Actualizados.xlsx
@@ -487,11 +487,11 @@
         <v>45958.45616898148</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>154.2269827722222</v>
+        <v>154.2519022959144</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>154 días, 05:26</t>
+          <t>154 días, 06:02</t>
         </is>
       </c>
     </row>
@@ -519,11 +519,11 @@
         <v>45959.70488425926</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>152.9782674944445</v>
+        <v>153.0031870181366</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>152 días, 23:28</t>
+          <t>153 días, 00:04</t>
         </is>
       </c>
     </row>
@@ -551,11 +551,11 @@
         <v>46092.63814814815</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>20.04500360555556</v>
+        <v>20.06992312924768</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>20 días, 01:04</t>
+          <t>20 días, 01:40</t>
         </is>
       </c>
     </row>
@@ -587,22 +587,22 @@
         <v>46099.61831018519</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>13.06484156851852</v>
+        <v>13.08976109221065</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>13 días, 01:33</t>
+          <t>13 días, 02:09</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>WO000032736</t>
+          <t>WO000032971</t>
         </is>
       </c>
       <c r="B6" s="1" t="n">
-        <v>46107.78501157407</v>
+        <v>46110.74581018519</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -616,65 +616,65 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BARRANQUILLA_CENTRO</t>
+          <t>SOLEDAD_SOLEDAD_2000</t>
         </is>
       </c>
       <c r="F6" s="1" t="n">
-        <v>46112.58827546296</v>
+        <v>46112.10444444444</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>0.09487629074074073</v>
+        <v>0.6036268329513889</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>0 días, 02:16</t>
+          <t>0 días, 14:29</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>WO000032775</t>
+          <t>WO000032974</t>
         </is>
       </c>
       <c r="B7" s="1" t="n">
-        <v>46108.39037037037</v>
+        <v>46110.79131944444</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>OYM_NOC_PROD</t>
+          <t>OYM_CAR_PROD</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ANTIOQUIA</t>
+          <t>ATLANTICO</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>MEDELLIN_ARANJUEZ</t>
+          <t>BARRANQUILLA_DELICIAS</t>
         </is>
       </c>
       <c r="F7" s="1" t="n">
-        <v>46112.34922453704</v>
+        <v>46112.11253472222</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>0.3339272166666666</v>
+        <v>0.5955365551736111</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>0 días, 08:00</t>
+          <t>0 días, 14:17</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>WO000032799</t>
+          <t>WO000032925</t>
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>46108.50020833333</v>
+        <v>46109.72104166666</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -692,61 +692,57 @@
         </is>
       </c>
       <c r="F8" s="1" t="n">
-        <v>46112.6127662037</v>
+        <v>46112.11261574074</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>0.07038555000000001</v>
+        <v>0.5954555366550927</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>0 días, 01:41</t>
+          <t>0 días, 14:17</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>WO000032900</t>
+          <t>WO000033020</t>
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>46109.52395833333</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>OYM_CAR_PROD</t>
-        </is>
-      </c>
+        <v>46111.57645833334</v>
+      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>ATLANTICO</t>
+          <t>ANTIOQUIA</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BARRANQUILLA_NUEVO_HORIZONTE</t>
+          <t>RIONEGRO_CENTRO</t>
         </is>
       </c>
       <c r="F9" s="1" t="n">
-        <v>46112.5987037037</v>
+        <v>46112.11642361111</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>0.08444805</v>
+        <v>0.5916476662847222</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>0 días, 02:01</t>
+          <t>0 días, 14:11</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>WO000032925</t>
+          <t>WO000032997</t>
         </is>
       </c>
       <c r="B10" s="1" t="n">
-        <v>46109.72104166666</v>
+        <v>46111.47408564815</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -764,97 +760,97 @@
         </is>
       </c>
       <c r="F10" s="1" t="n">
-        <v>46112.11261574074</v>
+        <v>46112.11672453704</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>0.570536012962963</v>
+        <v>0.5913467403587963</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>0 días, 13:41</t>
+          <t>0 días, 14:11</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>WO000032932</t>
+          <t>WO000033056</t>
         </is>
       </c>
       <c r="B11" s="1" t="n">
-        <v>46109.91506944445</v>
+        <v>46111.85439814815</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>OYM_CAR_PROD</t>
+          <t>OYM_BOG_SUR PROD</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>ATLANTICO</t>
+          <t>META</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BARRANQUILLA_NUEVO_HORIZONTE</t>
+          <t>ACACIAS_CENTRO</t>
         </is>
       </c>
       <c r="F11" s="1" t="n">
-        <v>46112.26559027778</v>
+        <v>46112.12311342593</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>0.417561475925926</v>
+        <v>0.5849578514699074</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>0 días, 10:01</t>
+          <t>0 días, 14:02</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>WO000032949</t>
+          <t>WO000033070</t>
         </is>
       </c>
       <c r="B12" s="1" t="n">
-        <v>46110.44939814815</v>
+        <v>46112.22738425926</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>OYM_CAR_PROD</t>
+          <t>OYM_BOG_SUR PROD</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>ATLANTICO</t>
+          <t>BOGOTA D.C</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BARRANQUILLA_NUEVO_HORIZONTE</t>
+          <t>FUSAGASUGA_CENTRO</t>
         </is>
       </c>
       <c r="F12" s="1" t="n">
-        <v>46112.42061342593</v>
+        <v>46112.22817129629</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>0.2625383277777777</v>
+        <v>0.479899981099537</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>0 días, 06:18</t>
+          <t>0 días, 11:31</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>WO000032958</t>
+          <t>WO000033060</t>
         </is>
       </c>
       <c r="B13" s="1" t="n">
-        <v>46110.55072916667</v>
+        <v>46112.02369212963</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -868,29 +864,29 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BARRANQUILLA_NUEVO_HORIZONTE</t>
+          <t>BARRANQUILLA_VICTORIA</t>
         </is>
       </c>
       <c r="F13" s="1" t="n">
-        <v>46112.62854166667</v>
+        <v>46112.2646875</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>0.05461008703703704</v>
+        <v>0.4433837773958333</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>0 días, 01:18</t>
+          <t>0 días, 10:38</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>WO000032971</t>
+          <t>WO000032932</t>
         </is>
       </c>
       <c r="B14" s="1" t="n">
-        <v>46110.74581018519</v>
+        <v>46109.91506944445</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -904,29 +900,29 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SOLEDAD_SOLEDAD_2000</t>
+          <t>BARRANQUILLA_NUEVO_HORIZONTE</t>
         </is>
       </c>
       <c r="F14" s="1" t="n">
-        <v>46112.10444444444</v>
+        <v>46112.26559027778</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>0.5787073092592593</v>
+        <v>0.4424809996180555</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>0 días, 13:53</t>
+          <t>0 días, 10:37</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>WO000032974</t>
+          <t>WO000033028</t>
         </is>
       </c>
       <c r="B15" s="1" t="n">
-        <v>46110.79131944444</v>
+        <v>46111.66822916667</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -940,65 +936,65 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BARRANQUILLA_DELICIAS</t>
+          <t>SOLEDAD_SOLEDAD_2000</t>
         </is>
       </c>
       <c r="F15" s="1" t="n">
-        <v>46112.11253472222</v>
+        <v>46112.2699074074</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>0.5706170314814815</v>
+        <v>0.4381638699884259</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>0 días, 13:41</t>
+          <t>0 días, 10:30</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>WO000032975</t>
+          <t>WO000032775</t>
         </is>
       </c>
       <c r="B16" s="1" t="n">
-        <v>46110.80520833333</v>
+        <v>46108.39037037037</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>OYM_CAR_PROD</t>
+          <t>OYM_NOC_PROD</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>ATLANTICO</t>
+          <t>ANTIOQUIA</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BARRANQUILLA_NUEVO_HORIZONTE</t>
+          <t>MEDELLIN_ARANJUEZ</t>
         </is>
       </c>
       <c r="F16" s="1" t="n">
-        <v>46112.59829861111</v>
+        <v>46112.34922453704</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>0.08485314259259259</v>
+        <v>0.3588467403587963</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>0 días, 02:02</t>
+          <t>0 días, 08:36</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>WO000032983</t>
+          <t>WO000032949</t>
         </is>
       </c>
       <c r="B17" s="1" t="n">
-        <v>46111.00909722222</v>
+        <v>46110.44939814815</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -1012,29 +1008,29 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BARRANQUILLA_CARIBE</t>
+          <t>BARRANQUILLA_NUEVO_HORIZONTE</t>
         </is>
       </c>
       <c r="F17" s="1" t="n">
-        <v>46112.50707175926</v>
+        <v>46112.42061342593</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>0.1760799944444444</v>
+        <v>0.2874578514699074</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>0 días, 04:13</t>
+          <t>0 días, 06:53</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>WO000032997</t>
+          <t>WO000033086</t>
         </is>
       </c>
       <c r="B18" s="1" t="n">
-        <v>46111.47408564815</v>
+        <v>46112.49396990741</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -1043,138 +1039,142 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>ATLANTICO</t>
+          <t>MAGDALENA</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BARRANQUILLA_NUEVO_HORIZONTE</t>
+          <t>SANTA_MARTA_SAN_PEDRO</t>
         </is>
       </c>
       <c r="F18" s="1" t="n">
-        <v>46112.11672453704</v>
+        <v>46112.50060185185</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>0.5664272166666667</v>
+        <v>0.2074694255439815</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>0 días, 13:35</t>
+          <t>0 días, 04:58</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>WO000033005</t>
+          <t>WO000032983</t>
         </is>
       </c>
       <c r="B19" s="1" t="n">
-        <v>46111.49688657407</v>
+        <v>46111.00909722222</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>OYM_CAR_SUR_PROD</t>
+          <t>OYM_CAR_PROD</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>CORDOBA</t>
+          <t>ATLANTICO</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>MONTERIA_LA_CASTELLANA</t>
+          <t>BARRANQUILLA_CARIBE</t>
         </is>
       </c>
       <c r="F19" s="1" t="n">
-        <v>46112.59883101852</v>
+        <v>46112.50707175926</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>0.08432073518518519</v>
+        <v>0.2009995181365741</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>0 días, 02:01</t>
+          <t>0 días, 04:49</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>WO000033018</t>
+          <t>WO000033089</t>
         </is>
       </c>
       <c r="B20" s="1" t="n">
-        <v>46111.56916666667</v>
+        <v>46112.52482638889</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>OYM_NOC_PROD</t>
+          <t>OYM_BOG_SUR PROD</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>ANTIOQUIA</t>
+          <t>META</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>RIONEGRO_CENTRO</t>
+          <t>VILLAVICENCIO_VILLA_ORTIZ</t>
         </is>
       </c>
       <c r="F20" s="1" t="n">
-        <v>46112.55466435185</v>
+        <v>46112.52521990741</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>0.1284874018518518</v>
+        <v>0.1828513699884259</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>0 días, 03:05</t>
+          <t>0 días, 04:23</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>WO000033020</t>
+          <t>WO000033090</t>
         </is>
       </c>
       <c r="B21" s="1" t="n">
-        <v>46111.57645833334</v>
-      </c>
-      <c r="C21" t="inlineStr"/>
+        <v>46112.52734953703</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>OYM_BOG_PROD</t>
+        </is>
+      </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>ANTIOQUIA</t>
+          <t>BOGOTA D.C</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>RIONEGRO_CENTRO</t>
+          <t>23106_LA_ESPANOLA</t>
         </is>
       </c>
       <c r="F21" s="1" t="n">
-        <v>46112.11642361111</v>
+        <v>46112.52790509259</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>0.5667281425925926</v>
+        <v>0.1801661848032408</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>0 días, 13:36</t>
+          <t>0 días, 04:19</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>WO000033028</t>
+          <t>WO000033095</t>
         </is>
       </c>
       <c r="B22" s="1" t="n">
-        <v>46111.66822916667</v>
+        <v>46112.5475</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1188,101 +1188,101 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SOLEDAD_SOLEDAD_2000</t>
+          <t>BARRANQUILLA_VICTORIA</t>
         </is>
       </c>
       <c r="F22" s="1" t="n">
-        <v>46112.2699074074</v>
+        <v>46112.54766203704</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>0.4132443462962963</v>
+        <v>0.1604092403587963</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>0 días, 09:55</t>
+          <t>0 días, 03:50</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>WO000033033</t>
+          <t>WO000033018</t>
         </is>
       </c>
       <c r="B23" s="1" t="n">
-        <v>46111.70326388889</v>
+        <v>46111.56916666667</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>OYM_SOC_PROD</t>
+          <t>OYM_NOC_PROD</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>VALLE DEL CAUCA</t>
+          <t>ANTIOQUIA</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>JAMUNDI_CENTRO</t>
+          <t>RIONEGRO_CENTRO</t>
         </is>
       </c>
       <c r="F23" s="1" t="n">
-        <v>46112.61951388889</v>
+        <v>46112.55466435185</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>0.06363786481481482</v>
+        <v>0.1534069255439815</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0 días, 01:31</t>
+          <t>0 días, 03:40</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>WO000033034</t>
+          <t>WO000033096</t>
         </is>
       </c>
       <c r="B24" s="1" t="n">
-        <v>46111.70519675926</v>
+        <v>46112.55680555556</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>OYM_EJE_CAF_PROD</t>
+          <t>OYM_CAR_PROD</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>QUINDIO</t>
+          <t>MAGDALENA</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>ARMENIA_SUR</t>
+          <t>SANTA_MARTA_SAN_PEDRO</t>
         </is>
       </c>
       <c r="F24" s="1" t="n">
-        <v>46112.60510416667</v>
+        <v>46112.56127314815</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>0.07804758703703704</v>
+        <v>0.1467981292476852</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>0 días, 01:52</t>
+          <t>0 días, 03:31</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>WO000033035</t>
+          <t>WO000033097</t>
         </is>
       </c>
       <c r="B25" s="1" t="n">
-        <v>46111.7149074074</v>
+        <v>46112.56569444444</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1296,249 +1296,249 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>BARRANQUILLA_CENTRO</t>
+          <t>BARRANQUILLA_VICTORIA</t>
         </is>
       </c>
       <c r="F25" s="1" t="n">
-        <v>46112.59583333333</v>
+        <v>46112.56730324074</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>0.08731842037037037</v>
+        <v>0.1407680366550926</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>0 días, 02:05</t>
+          <t>0 días, 03:22</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>WO000033036</t>
+          <t>WO000033048</t>
         </is>
       </c>
       <c r="B26" s="1" t="n">
-        <v>46111.71737268518</v>
+        <v>46111.77086805556</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>OYM_CAR_PROD</t>
+          <t>OYM_BOG_SUR PROD</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>ATLANTICO</t>
+          <t>META</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>BARRANQUILLA_VICTORIA</t>
+          <t>VILLAVICENCIO_VILLA_ORTIZ</t>
         </is>
       </c>
       <c r="F26" s="1" t="n">
-        <v>46112.58013888889</v>
+        <v>46112.57362268519</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>0.1030128648148148</v>
+        <v>0.1344485922106481</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>0 días, 02:28</t>
+          <t>0 días, 03:13</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>WO000033038</t>
+          <t>WO000033036</t>
         </is>
       </c>
       <c r="B27" s="1" t="n">
-        <v>46111.73001157407</v>
+        <v>46111.71737268518</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>OYM_SOC_PROD</t>
+          <t>OYM_CAR_PROD</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>VALLE DEL CAUCA</t>
+          <t>ATLANTICO</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>JAMUNDI_CENTRO</t>
+          <t>BARRANQUILLA_VICTORIA</t>
         </is>
       </c>
       <c r="F27" s="1" t="n">
-        <v>46112.63153935185</v>
+        <v>46112.58013888889</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>0.05161240185185186</v>
+        <v>0.1279323885069445</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>0 días, 01:14</t>
+          <t>0 días, 03:04</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>WO000033041</t>
+          <t>WO000033061</t>
         </is>
       </c>
       <c r="B28" s="1" t="n">
-        <v>46111.74322916667</v>
+        <v>46112.05803240741</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>OYM_CAR_PROD</t>
+          <t>OYM_BOG_SUR PROD</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>MAGDALENA</t>
+          <t>BOGOTA D.C</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SANTA_MARTA_CENTRO</t>
+          <t>SOACHA_CENTRO_DE_GRAVEDAD_1</t>
         </is>
       </c>
       <c r="F28" s="1" t="n">
-        <v>46112.62921296297</v>
+        <v>46112.58533564815</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>0.05393879074074074</v>
+        <v>0.1227356292476852</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>0 días, 01:17</t>
+          <t>0 días, 02:56</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>WO000033047</t>
+          <t>WO000032736</t>
         </is>
       </c>
       <c r="B29" s="1" t="n">
-        <v>46111.76734953704</v>
+        <v>46107.78501157407</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>OYM_BOG_CENTRO PROD</t>
+          <t>OYM_CAR_PROD</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>BOGOTA D.C</t>
+          <t>ATLANTICO</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>51261_TELECOM_CENTRO</t>
+          <t>BARRANQUILLA_CENTRO</t>
         </is>
       </c>
       <c r="F29" s="1" t="n">
-        <v>46112.6234375</v>
+        <v>46112.58827546296</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>0.05971425370370371</v>
+        <v>0.1197958144328704</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>0 días, 01:25</t>
+          <t>0 días, 02:52</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>WO000033048</t>
+          <t>WO000033087</t>
         </is>
       </c>
       <c r="B30" s="1" t="n">
-        <v>46111.77086805556</v>
+        <v>46112.51030092593</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>OYM_BOG_SUR PROD</t>
+          <t>OYM_CAR_PROD</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>ATLANTICO</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>VILLAVICENCIO_VILLA_ORTIZ</t>
+          <t>BARRANQUILLA_DELICIAS</t>
         </is>
       </c>
       <c r="F30" s="1" t="n">
-        <v>46112.57362268519</v>
+        <v>46112.59091435185</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>0.1095290685185185</v>
+        <v>0.1171569255439815</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>0 días, 02:37</t>
+          <t>0 días, 02:48</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>WO000033049</t>
+          <t>WO000033035</t>
         </is>
       </c>
       <c r="B31" s="1" t="n">
-        <v>46111.77138888889</v>
+        <v>46111.7149074074</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>OYM_SOC_PROD</t>
+          <t>OYM_CAR_PROD</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>VALLE DEL CAUCA</t>
+          <t>ATLANTICO</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>JAMUNDI_CENTRO</t>
+          <t>BARRANQUILLA_CENTRO</t>
         </is>
       </c>
       <c r="F31" s="1" t="n">
-        <v>46112.61924768519</v>
+        <v>46112.59583333333</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>0.06390406851851851</v>
+        <v>0.1122379440625</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>0 días, 01:32</t>
+          <t>0 días, 02:41</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>WO000033050</t>
+          <t>WO000033098</t>
         </is>
       </c>
       <c r="B32" s="1" t="n">
-        <v>46111.773125</v>
+        <v>46112.57793981482</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>OYM_BOG_SUR PROD</t>
+          <t>OYM_BOG_PROD</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1548,65 +1548,65 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>51000_PROGRESO</t>
+          <t>23106_LA_ESPANOLA</t>
         </is>
       </c>
       <c r="F32" s="1" t="n">
-        <v>46112.62898148148</v>
+        <v>46112.59709490741</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>0.05417027222222223</v>
+        <v>0.1109763699884259</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>0 días, 01:18</t>
+          <t>0 días, 02:39</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>WO000033056</t>
+          <t>WO000032975</t>
         </is>
       </c>
       <c r="B33" s="1" t="n">
-        <v>46111.85439814815</v>
+        <v>46110.80520833333</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>OYM_BOG_SUR PROD</t>
+          <t>OYM_CAR_PROD</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>ATLANTICO</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>ACACIAS_CENTRO</t>
+          <t>BARRANQUILLA_NUEVO_HORIZONTE</t>
         </is>
       </c>
       <c r="F33" s="1" t="n">
-        <v>46112.12311342593</v>
+        <v>46112.59829861111</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>0.5600383277777778</v>
+        <v>0.1097726662847222</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>0 días, 13:26</t>
+          <t>0 días, 02:38</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>WO000033060</t>
+          <t>WO000032900</t>
         </is>
       </c>
       <c r="B34" s="1" t="n">
-        <v>46112.02369212963</v>
+        <v>46109.52395833333</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1620,137 +1620,137 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>BARRANQUILLA_VICTORIA</t>
+          <t>BARRANQUILLA_NUEVO_HORIZONTE</t>
         </is>
       </c>
       <c r="F34" s="1" t="n">
-        <v>46112.2646875</v>
+        <v>46112.5987037037</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>0.4184642537037037</v>
+        <v>0.1093675736921296</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>0 días, 10:02</t>
+          <t>0 días, 02:37</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>WO000033061</t>
+          <t>WO000033005</t>
         </is>
       </c>
       <c r="B35" s="1" t="n">
-        <v>46112.05803240741</v>
+        <v>46111.49688657407</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>OYM_BOG_SUR PROD</t>
+          <t>OYM_CAR_SUR_PROD</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>BOGOTA D.C</t>
+          <t>CORDOBA</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SOACHA_CENTRO_DE_GRAVEDAD_1</t>
+          <t>MONTERIA_LA_CASTELLANA</t>
         </is>
       </c>
       <c r="F35" s="1" t="n">
-        <v>46112.58533564815</v>
+        <v>46112.59883101852</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>0.09781610555555555</v>
+        <v>0.1092402588773148</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>0 días, 02:20</t>
+          <t>0 días, 02:37</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>WO000033063</t>
+          <t>WO000033034</t>
         </is>
       </c>
       <c r="B36" s="1" t="n">
-        <v>46112.07569444444</v>
+        <v>46111.70519675926</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>OYM_CAR_PROD</t>
+          <t>OYM_EJE_CAF_PROD</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>ATLANTICO</t>
+          <t>QUINDIO</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>BARRANQUILLA_VICTORIA</t>
+          <t>ARMENIA_SUR</t>
         </is>
       </c>
       <c r="F36" s="1" t="n">
-        <v>46112.61540509259</v>
+        <v>46112.60510416667</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>0.06774666111111112</v>
+        <v>0.1029671107291667</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>0 días, 01:37</t>
+          <t>0 días, 02:28</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>WO000033068</t>
+          <t>WO000033088</t>
         </is>
       </c>
       <c r="B37" s="1" t="n">
-        <v>46112.1821875</v>
+        <v>46112.51873842593</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>OYM_SOC_PROD</t>
+          <t>OYM_BOG_CENTRO PROD</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>VALLE DEL CAUCA</t>
+          <t>BOGOTA D.C</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>PALMIRA_CENTRO</t>
+          <t>FUNZA_CENTRO</t>
         </is>
       </c>
       <c r="F37" s="1" t="n">
-        <v>46112.61197916666</v>
+        <v>46112.6057175926</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>0.07117258703703704</v>
+        <v>0.1023536848032408</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>0 días, 01:42</t>
+          <t>0 días, 02:27</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>WO000033070</t>
+          <t>WO000033092</t>
         </is>
       </c>
       <c r="B38" s="1" t="n">
-        <v>46112.22738425926</v>
+        <v>46112.53222222222</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1764,65 +1764,65 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>FUSAGASUGA_CENTRO</t>
+          <t>SOACHA_CENTRO_DE_GRAVEDAD_1</t>
         </is>
       </c>
       <c r="F38" s="1" t="n">
-        <v>46112.22817129629</v>
+        <v>46112.61043981482</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>0.4549804574074074</v>
+        <v>0.09763146258101853</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>0 días, 10:55</t>
+          <t>0 días, 02:20</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>WO000033075</t>
+          <t>WO000033068</t>
         </is>
       </c>
       <c r="B39" s="1" t="n">
-        <v>46112.36907407407</v>
+        <v>46112.1821875</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>OYM_BOG_SUR PROD</t>
+          <t>OYM_SOC_PROD</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>BOGOTA D.C</t>
+          <t>VALLE DEL CAUCA</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>FUSAGASUGA_CENTRO</t>
+          <t>PALMIRA_CENTRO</t>
         </is>
       </c>
       <c r="F39" s="1" t="n">
-        <v>46112.63113425926</v>
+        <v>46112.61197916666</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>0.05201749444444444</v>
+        <v>0.09609211072916668</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>0 días, 01:14</t>
+          <t>0 días, 02:18</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>WO000033080</t>
+          <t>WO000032799</t>
         </is>
       </c>
       <c r="B40" s="1" t="n">
-        <v>46112.4299537037</v>
+        <v>46108.50020833333</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1831,394 +1831,394 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>CESAR</t>
+          <t>ATLANTICO</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>VALLEDUPAR_ESPERANZA</t>
+          <t>BARRANQUILLA_NUEVO_HORIZONTE</t>
         </is>
       </c>
       <c r="F40" s="1" t="n">
-        <v>46112.63335648148</v>
+        <v>46112.6127662037</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>0.04979527222222222</v>
+        <v>0.09530507369212964</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>0 días, 01:11</t>
+          <t>0 días, 02:17</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>WO000033081</t>
+          <t>WO000033063</t>
         </is>
       </c>
       <c r="B41" s="1" t="n">
-        <v>46112.43398148148</v>
+        <v>46112.07569444444</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>OYM_BOG_PROD</t>
+          <t>OYM_CAR_PROD</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>BOGOTA D.C</t>
+          <t>ATLANTICO</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>CHIA_MATRIZ</t>
+          <t>BARRANQUILLA_VICTORIA</t>
         </is>
       </c>
       <c r="F41" s="1" t="n">
-        <v>46112.6209837963</v>
+        <v>46112.61540509259</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>0.06216795740740741</v>
+        <v>0.09266618480324074</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>0 días, 01:29</t>
+          <t>0 días, 02:13</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>WO000033082</t>
+          <t>WO000033100</t>
         </is>
       </c>
       <c r="B42" s="1" t="n">
-        <v>46112.45357638889</v>
+        <v>46112.61635416667</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>OYM_CAR_PROD</t>
+          <t>OYM_NOC_PROD</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>ATLANTICO</t>
+          <t>ANTIOQUIA</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>BARRANQUILLA_SAN_FRANCISCO</t>
+          <t>MEDELLIN_ARANJUEZ</t>
         </is>
       </c>
       <c r="F42" s="1" t="n">
-        <v>46112.63296296296</v>
+        <v>46112.61690972222</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>0.05018879074074074</v>
+        <v>0.0911615551736111</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>0 días, 01:12</t>
+          <t>0 días, 02:11</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>WO000033086</t>
+          <t>WO000033049</t>
         </is>
       </c>
       <c r="B43" s="1" t="n">
-        <v>46112.49396990741</v>
+        <v>46111.77138888889</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>OYM_CAR_PROD</t>
+          <t>OYM_SOC_PROD</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>MAGDALENA</t>
+          <t>VALLE DEL CAUCA</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>SANTA_MARTA_SAN_PEDRO</t>
+          <t>JAMUNDI_CENTRO</t>
         </is>
       </c>
       <c r="F43" s="1" t="n">
-        <v>46112.50060185185</v>
+        <v>46112.61924768519</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>0.1825499018518519</v>
+        <v>0.08882359221064814</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>0 días, 04:22</t>
+          <t>0 días, 02:07</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>WO000033087</t>
+          <t>WO000033033</t>
         </is>
       </c>
       <c r="B44" s="1" t="n">
-        <v>46112.51030092593</v>
+        <v>46111.70326388889</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>OYM_CAR_PROD</t>
+          <t>OYM_SOC_PROD</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>ATLANTICO</t>
+          <t>VALLE DEL CAUCA</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>BARRANQUILLA_DELICIAS</t>
+          <t>JAMUNDI_CENTRO</t>
         </is>
       </c>
       <c r="F44" s="1" t="n">
-        <v>46112.59091435185</v>
+        <v>46112.61951388889</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>0.09223740185185185</v>
+        <v>0.08855738850694445</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>0 días, 02:12</t>
+          <t>0 días, 02:07</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>WO000033088</t>
+          <t>WO000033101</t>
         </is>
       </c>
       <c r="B45" s="1" t="n">
-        <v>46112.51873842593</v>
+        <v>46112.61912037037</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>OYM_BOG_CENTRO PROD</t>
+          <t>OYM_CAR_PROD</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>BOGOTA D.C</t>
+          <t>ATLANTICO</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>FUNZA_CENTRO</t>
+          <t>BARRANQUILLA_VICTORIA</t>
         </is>
       </c>
       <c r="F45" s="1" t="n">
-        <v>46112.6057175926</v>
+        <v>46112.61989583333</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>0.07743416111111111</v>
+        <v>0.0881754440625</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>0 días, 01:51</t>
+          <t>0 días, 02:06</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>WO000033089</t>
+          <t>WO000033081</t>
         </is>
       </c>
       <c r="B46" s="1" t="n">
-        <v>46112.52482638889</v>
+        <v>46112.43398148148</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>OYM_BOG_SUR PROD</t>
+          <t>OYM_BOG_PROD</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>BOGOTA D.C</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>VILLAVICENCIO_VILLA_ORTIZ</t>
+          <t>CHIA_MATRIZ</t>
         </is>
       </c>
       <c r="F46" s="1" t="n">
-        <v>46112.52521990741</v>
+        <v>46112.6209837963</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>0.1579318462962963</v>
+        <v>0.08708748109953704</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>0 días, 03:47</t>
+          <t>0 días, 02:05</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>WO000033090</t>
+          <t>WO000033103</t>
         </is>
       </c>
       <c r="B47" s="1" t="n">
-        <v>46112.52734953703</v>
+        <v>46112.62123842593</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>OYM_BOG_PROD</t>
+          <t>OYM_CAR_PROD</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>BOGOTA D.C</t>
+          <t>ATLANTICO</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>23106_LA_ESPANOLA</t>
+          <t>PUERTO_COLOMBIA_CENTRO</t>
         </is>
       </c>
       <c r="F47" s="1" t="n">
-        <v>46112.52790509259</v>
+        <v>46112.62127314815</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>0.1552466611111111</v>
+        <v>0.08679812924768518</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>0 días, 03:43</t>
+          <t>0 días, 02:04</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>WO000033092</t>
+          <t>WO000033104</t>
         </is>
       </c>
       <c r="B48" s="1" t="n">
-        <v>46112.53222222222</v>
+        <v>46112.62290509259</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>OYM_BOG_SUR PROD</t>
+          <t>OYM_CAR_PROD</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>BOGOTA D.C</t>
+          <t>ATLANTICO</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>SOACHA_CENTRO_DE_GRAVEDAD_1</t>
+          <t>BARRANQUILLA_VICTORIA</t>
         </is>
       </c>
       <c r="F48" s="1" t="n">
-        <v>46112.61043981482</v>
+        <v>46112.62322916667</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>0.0727119388888889</v>
+        <v>0.08484211072916667</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>0 días, 01:44</t>
+          <t>0 días, 02:02</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>WO000033093</t>
+          <t>WO000033047</t>
         </is>
       </c>
       <c r="B49" s="1" t="n">
-        <v>46112.53445601852</v>
+        <v>46111.76734953704</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>OYM_SOC_PROD</t>
+          <t>OYM_BOG_CENTRO PROD</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>VALLE DEL CAUCA</t>
+          <t>BOGOTA D.C</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>CALI_VALLE_DE_LILI</t>
+          <t>51261_TELECOM_CENTRO</t>
         </is>
       </c>
       <c r="F49" s="1" t="n">
-        <v>46112.63163194444</v>
+        <v>46112.6234375</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>0.05151980925925926</v>
+        <v>0.08463377739583333</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>0 días, 01:14</t>
+          <t>0 días, 02:01</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>WO000033095</t>
+          <t>WO000033105</t>
         </is>
       </c>
       <c r="B50" s="1" t="n">
-        <v>46112.5475</v>
+        <v>46112.62443287037</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>OYM_CAR_PROD</t>
+          <t>OYM_BOG_SUR PROD</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>ATLANTICO</t>
+          <t>META</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>BARRANQUILLA_VICTORIA</t>
+          <t>VILLAVICENCIO_CENTRO</t>
         </is>
       </c>
       <c r="F50" s="1" t="n">
-        <v>46112.54766203704</v>
+        <v>46112.62462962963</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>0.1354897166666666</v>
+        <v>0.08344164776620371</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>0 días, 03:15</t>
+          <t>0 días, 02:00</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>WO000033096</t>
+          <t>WO000032958</t>
         </is>
       </c>
       <c r="B51" s="1" t="n">
-        <v>46112.55680555556</v>
+        <v>46110.55072916667</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -2227,74 +2227,74 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>MAGDALENA</t>
+          <t>ATLANTICO</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>SANTA_MARTA_SAN_PEDRO</t>
+          <t>BARRANQUILLA_NUEVO_HORIZONTE</t>
         </is>
       </c>
       <c r="F51" s="1" t="n">
-        <v>46112.56127314815</v>
+        <v>46112.62854166667</v>
       </c>
       <c r="G51" s="2" t="n">
-        <v>0.1218786055555555</v>
+        <v>0.07952961072916666</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>0 días, 02:55</t>
+          <t>0 días, 01:54</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>WO000033097</t>
+          <t>WO000033106</t>
         </is>
       </c>
       <c r="B52" s="1" t="n">
-        <v>46112.56569444444</v>
+        <v>46112.62850694444</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>OYM_CAR_PROD</t>
+          <t>OYM_BOG_PROD</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>ATLANTICO</t>
+          <t>BOGOTA D.C</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>BARRANQUILLA_VICTORIA</t>
+          <t>11000_AUTOPISTA</t>
         </is>
       </c>
       <c r="F52" s="1" t="n">
-        <v>46112.56730324074</v>
+        <v>46112.62855324074</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>0.115848512962963</v>
+        <v>0.07951803665509259</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>0 días, 02:46</t>
+          <t>0 días, 01:54</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>WO000033098</t>
+          <t>WO000033050</t>
         </is>
       </c>
       <c r="B53" s="1" t="n">
-        <v>46112.57793981482</v>
+        <v>46111.773125</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>OYM_BOG_PROD</t>
+          <t>OYM_BOG_SUR PROD</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2304,234 +2304,234 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>23106_LA_ESPANOLA</t>
+          <t>51000_PROGRESO</t>
         </is>
       </c>
       <c r="F53" s="1" t="n">
-        <v>46112.59709490741</v>
+        <v>46112.62898148148</v>
       </c>
       <c r="G53" s="2" t="n">
-        <v>0.0860568462962963</v>
+        <v>0.07908979591435185</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>0 días, 02:03</t>
+          <t>0 días, 01:53</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>WO000033100</t>
+          <t>WO000033041</t>
         </is>
       </c>
       <c r="B54" s="1" t="n">
-        <v>46112.61635416667</v>
+        <v>46111.74322916667</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>OYM_NOC_PROD</t>
+          <t>OYM_CAR_PROD</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>ANTIOQUIA</t>
+          <t>MAGDALENA</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>MEDELLIN_ARANJUEZ</t>
+          <t>SANTA_MARTA_CENTRO</t>
         </is>
       </c>
       <c r="F54" s="1" t="n">
-        <v>46112.61690972222</v>
+        <v>46112.62921296297</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>0.06624203148148149</v>
+        <v>0.07885831443287036</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>0 días, 01:35</t>
+          <t>0 días, 01:53</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>WO000033101</t>
+          <t>WO000033075</t>
         </is>
       </c>
       <c r="B55" s="1" t="n">
-        <v>46112.61912037037</v>
+        <v>46112.36907407407</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>OYM_CAR_PROD</t>
+          <t>OYM_BOG_SUR PROD</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>ATLANTICO</t>
+          <t>BOGOTA D.C</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>BARRANQUILLA_VICTORIA</t>
+          <t>FUSAGASUGA_CENTRO</t>
         </is>
       </c>
       <c r="F55" s="1" t="n">
-        <v>46112.61989583333</v>
+        <v>46112.63113425926</v>
       </c>
       <c r="G55" s="2" t="n">
-        <v>0.06325592037037037</v>
+        <v>0.07693701813657407</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>0 días, 01:31</t>
+          <t>0 días, 01:50</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>WO000033103</t>
+          <t>WO000033038</t>
         </is>
       </c>
       <c r="B56" s="1" t="n">
-        <v>46112.62123842593</v>
+        <v>46111.73001157407</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>OYM_CAR_PROD</t>
+          <t>OYM_SOC_PROD</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>ATLANTICO</t>
+          <t>VALLE DEL CAUCA</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>PUERTO_COLOMBIA_CENTRO</t>
+          <t>JAMUNDI_CENTRO</t>
         </is>
       </c>
       <c r="F56" s="1" t="n">
-        <v>46112.62127314815</v>
+        <v>46112.63153935185</v>
       </c>
       <c r="G56" s="2" t="n">
-        <v>0.06187860555555556</v>
+        <v>0.07653192554398149</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>0 días, 01:29</t>
+          <t>0 días, 01:50</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>WO000033104</t>
+          <t>WO000033093</t>
         </is>
       </c>
       <c r="B57" s="1" t="n">
-        <v>46112.62290509259</v>
+        <v>46112.53445601852</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>OYM_CAR_PROD</t>
+          <t>OYM_SOC_PROD</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>ATLANTICO</t>
+          <t>VALLE DEL CAUCA</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>BARRANQUILLA_VICTORIA</t>
+          <t>CALI_VALLE_DE_LILI</t>
         </is>
       </c>
       <c r="F57" s="1" t="n">
-        <v>46112.62322916667</v>
+        <v>46112.63163194444</v>
       </c>
       <c r="G57" s="2" t="n">
-        <v>0.05992258703703704</v>
+        <v>0.07643933295138888</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>0 días, 01:26</t>
+          <t>0 días, 01:50</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>WO000033105</t>
+          <t>WO000033082</t>
         </is>
       </c>
       <c r="B58" s="1" t="n">
-        <v>46112.62443287037</v>
+        <v>46112.45357638889</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>OYM_BOG_SUR PROD</t>
+          <t>OYM_CAR_PROD</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>ATLANTICO</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>VILLAVICENCIO_CENTRO</t>
+          <t>BARRANQUILLA_SAN_FRANCISCO</t>
         </is>
       </c>
       <c r="F58" s="1" t="n">
-        <v>46112.62462962963</v>
+        <v>46112.63296296296</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>0.05852212407407408</v>
+        <v>0.07510831443287037</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>0 días, 01:24</t>
+          <t>0 días, 01:48</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>WO000033106</t>
+          <t>WO000033080</t>
         </is>
       </c>
       <c r="B59" s="1" t="n">
-        <v>46112.62850694444</v>
+        <v>46112.4299537037</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>OYM_BOG_PROD</t>
+          <t>OYM_CAR_PROD</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>BOGOTA D.C</t>
+          <t>CESAR</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>11000_AUTOPISTA</t>
+          <t>VALLEDUPAR_ESPERANZA</t>
         </is>
       </c>
       <c r="F59" s="1" t="n">
-        <v>46112.62855324074</v>
+        <v>46112.63335648148</v>
       </c>
       <c r="G59" s="2" t="n">
-        <v>0.05459851296296297</v>
+        <v>0.07471479591435184</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>0 días, 01:18</t>
+          <t>0 días, 01:47</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(BarridoOne): :sparkles: Agrega el modulo para enviar el informe por un grupo de whats
</commit_message>
<xml_diff>
--- a/assets/Informe_Tiempos_Actualizados.xlsx
+++ b/assets/Informe_Tiempos_Actualizados.xlsx
@@ -487,11 +487,11 @@
         <v>45958.45616898148</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>154.2519022959144</v>
+        <v>154.9001869327662</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>154 días, 06:02</t>
+          <t>154 días, 21:36</t>
         </is>
       </c>
     </row>
@@ -519,11 +519,11 @@
         <v>45959.70488425926</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>153.0031870181366</v>
+        <v>153.6514716549884</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>153 días, 00:04</t>
+          <t>153 días, 15:38</t>
         </is>
       </c>
     </row>
@@ -551,11 +551,11 @@
         <v>46092.63814814815</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>20.06992312924768</v>
+        <v>20.71820776609954</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>20 días, 01:40</t>
+          <t>20 días, 17:14</t>
         </is>
       </c>
     </row>
@@ -587,11 +587,11 @@
         <v>46099.61831018519</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>13.08976109221065</v>
+        <v>13.7380457290625</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>13 días, 02:09</t>
+          <t>13 días, 17:42</t>
         </is>
       </c>
     </row>
@@ -623,11 +623,11 @@
         <v>46112.10444444444</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>0.6036268329513889</v>
+        <v>1.251911469803241</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>0 días, 14:29</t>
+          <t>1 días, 06:02</t>
         </is>
       </c>
     </row>
@@ -659,11 +659,11 @@
         <v>46112.11253472222</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>0.5955365551736111</v>
+        <v>1.243821192025463</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>0 días, 14:17</t>
+          <t>1 días, 05:51</t>
         </is>
       </c>
     </row>
@@ -695,11 +695,11 @@
         <v>46112.11261574074</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>0.5954555366550927</v>
+        <v>1.243740173506944</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>0 días, 14:17</t>
+          <t>1 días, 05:50</t>
         </is>
       </c>
     </row>
@@ -727,11 +727,11 @@
         <v>46112.11642361111</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>0.5916476662847222</v>
+        <v>1.239932303136574</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>0 días, 14:11</t>
+          <t>1 días, 05:45</t>
         </is>
       </c>
     </row>
@@ -763,11 +763,11 @@
         <v>46112.11672453704</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>0.5913467403587963</v>
+        <v>1.239631377210648</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>0 días, 14:11</t>
+          <t>1 días, 05:45</t>
         </is>
       </c>
     </row>
@@ -799,11 +799,11 @@
         <v>46112.12311342593</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>0.5849578514699074</v>
+        <v>1.233242488321759</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>0 días, 14:02</t>
+          <t>1 días, 05:35</t>
         </is>
       </c>
     </row>
@@ -835,11 +835,11 @@
         <v>46112.22817129629</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>0.479899981099537</v>
+        <v>1.128184617951389</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>0 días, 11:31</t>
+          <t>1 días, 03:04</t>
         </is>
       </c>
     </row>
@@ -871,11 +871,11 @@
         <v>46112.2646875</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>0.4433837773958333</v>
+        <v>1.091668414247685</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>0 días, 10:38</t>
+          <t>1 días, 02:12</t>
         </is>
       </c>
     </row>
@@ -907,11 +907,11 @@
         <v>46112.26559027778</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>0.4424809996180555</v>
+        <v>1.090765636469907</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>0 días, 10:37</t>
+          <t>1 días, 02:10</t>
         </is>
       </c>
     </row>
@@ -943,11 +943,11 @@
         <v>46112.2699074074</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>0.4381638699884259</v>
+        <v>1.086448506840278</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>0 días, 10:30</t>
+          <t>1 días, 02:04</t>
         </is>
       </c>
     </row>
@@ -979,11 +979,11 @@
         <v>46112.34922453704</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>0.3588467403587963</v>
+        <v>1.007131377210648</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>0 días, 08:36</t>
+          <t>1 días, 00:10</t>
         </is>
       </c>
     </row>
@@ -1015,11 +1015,11 @@
         <v>46112.42061342593</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>0.2874578514699074</v>
+        <v>0.9357424883217593</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>0 días, 06:53</t>
+          <t>0 días, 22:27</t>
         </is>
       </c>
     </row>
@@ -1051,11 +1051,11 @@
         <v>46112.50060185185</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>0.2074694255439815</v>
+        <v>0.8557540623958334</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>0 días, 04:58</t>
+          <t>0 días, 20:32</t>
         </is>
       </c>
     </row>
@@ -1087,11 +1087,11 @@
         <v>46112.50707175926</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>0.2009995181365741</v>
+        <v>0.8492841549884259</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>0 días, 04:49</t>
+          <t>0 días, 20:22</t>
         </is>
       </c>
     </row>
@@ -1123,11 +1123,11 @@
         <v>46112.52521990741</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>0.1828513699884259</v>
+        <v>0.8311360068402778</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>0 días, 04:23</t>
+          <t>0 días, 19:56</t>
         </is>
       </c>
     </row>
@@ -1159,11 +1159,11 @@
         <v>46112.52790509259</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>0.1801661848032408</v>
+        <v>0.8284508216550927</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>0 días, 04:19</t>
+          <t>0 días, 19:52</t>
         </is>
       </c>
     </row>
@@ -1195,11 +1195,11 @@
         <v>46112.54766203704</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>0.1604092403587963</v>
+        <v>0.8086938772106482</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>0 días, 03:50</t>
+          <t>0 días, 19:24</t>
         </is>
       </c>
     </row>
@@ -1231,11 +1231,11 @@
         <v>46112.55466435185</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>0.1534069255439815</v>
+        <v>0.8016915623958334</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0 días, 03:40</t>
+          <t>0 días, 19:14</t>
         </is>
       </c>
     </row>
@@ -1267,11 +1267,11 @@
         <v>46112.56127314815</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>0.1467981292476852</v>
+        <v>0.7950827660995371</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>0 días, 03:31</t>
+          <t>0 días, 19:04</t>
         </is>
       </c>
     </row>
@@ -1303,11 +1303,11 @@
         <v>46112.56730324074</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>0.1407680366550926</v>
+        <v>0.7890526735069445</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>0 días, 03:22</t>
+          <t>0 días, 18:56</t>
         </is>
       </c>
     </row>
@@ -1339,11 +1339,11 @@
         <v>46112.57362268519</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>0.1344485922106481</v>
+        <v>0.7827332290625</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>0 días, 03:13</t>
+          <t>0 días, 18:47</t>
         </is>
       </c>
     </row>
@@ -1375,11 +1375,11 @@
         <v>46112.58013888889</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>0.1279323885069445</v>
+        <v>0.7762170253587963</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>0 días, 03:04</t>
+          <t>0 días, 18:37</t>
         </is>
       </c>
     </row>
@@ -1411,11 +1411,11 @@
         <v>46112.58533564815</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>0.1227356292476852</v>
+        <v>0.7710202660995371</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>0 días, 02:56</t>
+          <t>0 días, 18:30</t>
         </is>
       </c>
     </row>
@@ -1447,11 +1447,11 @@
         <v>46112.58827546296</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>0.1197958144328704</v>
+        <v>0.7680804512847222</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>0 días, 02:52</t>
+          <t>0 días, 18:26</t>
         </is>
       </c>
     </row>
@@ -1483,11 +1483,11 @@
         <v>46112.59091435185</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>0.1171569255439815</v>
+        <v>0.7654415623958334</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>0 días, 02:48</t>
+          <t>0 días, 18:22</t>
         </is>
       </c>
     </row>
@@ -1519,11 +1519,11 @@
         <v>46112.59583333333</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>0.1122379440625</v>
+        <v>0.7605225809143519</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>0 días, 02:41</t>
+          <t>0 días, 18:15</t>
         </is>
       </c>
     </row>
@@ -1555,11 +1555,11 @@
         <v>46112.59709490741</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>0.1109763699884259</v>
+        <v>0.7592610068402778</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>0 días, 02:39</t>
+          <t>0 días, 18:13</t>
         </is>
       </c>
     </row>
@@ -1591,11 +1591,11 @@
         <v>46112.59829861111</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>0.1097726662847222</v>
+        <v>0.758057303136574</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>0 días, 02:38</t>
+          <t>0 días, 18:11</t>
         </is>
       </c>
     </row>
@@ -1627,11 +1627,11 @@
         <v>46112.5987037037</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>0.1093675736921296</v>
+        <v>0.7576522105439815</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>0 días, 02:37</t>
+          <t>0 días, 18:11</t>
         </is>
       </c>
     </row>
@@ -1663,11 +1663,11 @@
         <v>46112.59883101852</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>0.1092402588773148</v>
+        <v>0.7575248957291667</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>0 días, 02:37</t>
+          <t>0 días, 18:10</t>
         </is>
       </c>
     </row>
@@ -1699,11 +1699,11 @@
         <v>46112.60510416667</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>0.1029671107291667</v>
+        <v>0.7512517475810185</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>0 días, 02:28</t>
+          <t>0 días, 18:01</t>
         </is>
       </c>
     </row>
@@ -1735,11 +1735,11 @@
         <v>46112.6057175926</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>0.1023536848032408</v>
+        <v>0.7506383216550926</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>0 días, 02:27</t>
+          <t>0 días, 18:00</t>
         </is>
       </c>
     </row>
@@ -1771,11 +1771,11 @@
         <v>46112.61043981482</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>0.09763146258101853</v>
+        <v>0.7459160994328704</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>0 días, 02:20</t>
+          <t>0 días, 17:54</t>
         </is>
       </c>
     </row>
@@ -1807,11 +1807,11 @@
         <v>46112.61197916666</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>0.09609211072916668</v>
+        <v>0.7443767475810186</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>0 días, 02:18</t>
+          <t>0 días, 17:51</t>
         </is>
       </c>
     </row>
@@ -1843,11 +1843,11 @@
         <v>46112.6127662037</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>0.09530507369212964</v>
+        <v>0.7435897105439815</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>0 días, 02:17</t>
+          <t>0 días, 17:50</t>
         </is>
       </c>
     </row>
@@ -1879,11 +1879,11 @@
         <v>46112.61540509259</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>0.09266618480324074</v>
+        <v>0.7409508216550926</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>0 días, 02:13</t>
+          <t>0 días, 17:46</t>
         </is>
       </c>
     </row>
@@ -1915,11 +1915,11 @@
         <v>46112.61690972222</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>0.0911615551736111</v>
+        <v>0.739446192025463</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>0 días, 02:11</t>
+          <t>0 días, 17:44</t>
         </is>
       </c>
     </row>
@@ -1951,11 +1951,11 @@
         <v>46112.61924768519</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>0.08882359221064814</v>
+        <v>0.7371082290625001</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>0 días, 02:07</t>
+          <t>0 días, 17:41</t>
         </is>
       </c>
     </row>
@@ -1987,11 +1987,11 @@
         <v>46112.61951388889</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>0.08855738850694445</v>
+        <v>0.7368420253587963</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>0 días, 02:07</t>
+          <t>0 días, 17:41</t>
         </is>
       </c>
     </row>
@@ -2023,11 +2023,11 @@
         <v>46112.61989583333</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>0.0881754440625</v>
+        <v>0.7364600809143519</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>0 días, 02:06</t>
+          <t>0 días, 17:40</t>
         </is>
       </c>
     </row>
@@ -2059,11 +2059,11 @@
         <v>46112.6209837963</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>0.08708748109953704</v>
+        <v>0.7353721179513889</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>0 días, 02:05</t>
+          <t>0 días, 17:38</t>
         </is>
       </c>
     </row>
@@ -2095,11 +2095,11 @@
         <v>46112.62127314815</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>0.08679812924768518</v>
+        <v>0.735082766099537</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>0 días, 02:04</t>
+          <t>0 días, 17:38</t>
         </is>
       </c>
     </row>
@@ -2131,11 +2131,11 @@
         <v>46112.62322916667</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>0.08484211072916667</v>
+        <v>0.7331267475810186</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>0 días, 02:02</t>
+          <t>0 días, 17:35</t>
         </is>
       </c>
     </row>
@@ -2167,11 +2167,11 @@
         <v>46112.6234375</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>0.08463377739583333</v>
+        <v>0.7329184142476852</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>0 días, 02:01</t>
+          <t>0 días, 17:35</t>
         </is>
       </c>
     </row>
@@ -2203,11 +2203,11 @@
         <v>46112.62462962963</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>0.08344164776620371</v>
+        <v>0.7317262846180556</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>0 días, 02:00</t>
+          <t>0 días, 17:33</t>
         </is>
       </c>
     </row>
@@ -2239,11 +2239,11 @@
         <v>46112.62854166667</v>
       </c>
       <c r="G51" s="2" t="n">
-        <v>0.07952961072916666</v>
+        <v>0.7278142475810185</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>0 días, 01:54</t>
+          <t>0 días, 17:28</t>
         </is>
       </c>
     </row>
@@ -2275,11 +2275,11 @@
         <v>46112.62855324074</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>0.07951803665509259</v>
+        <v>0.7278026735069445</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>0 días, 01:54</t>
+          <t>0 días, 17:28</t>
         </is>
       </c>
     </row>
@@ -2311,11 +2311,11 @@
         <v>46112.62898148148</v>
       </c>
       <c r="G53" s="2" t="n">
-        <v>0.07908979591435185</v>
+        <v>0.7273744327662037</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>0 días, 01:53</t>
+          <t>0 días, 17:27</t>
         </is>
       </c>
     </row>
@@ -2347,11 +2347,11 @@
         <v>46112.62921296297</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>0.07885831443287036</v>
+        <v>0.7271429512847223</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>0 días, 01:53</t>
+          <t>0 días, 17:27</t>
         </is>
       </c>
     </row>
@@ -2383,11 +2383,11 @@
         <v>46112.63113425926</v>
       </c>
       <c r="G55" s="2" t="n">
-        <v>0.07693701813657407</v>
+        <v>0.7252216549884259</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>0 días, 01:50</t>
+          <t>0 días, 17:24</t>
         </is>
       </c>
     </row>
@@ -2419,11 +2419,11 @@
         <v>46112.63153935185</v>
       </c>
       <c r="G56" s="2" t="n">
-        <v>0.07653192554398149</v>
+        <v>0.7248165623958334</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>0 días, 01:50</t>
+          <t>0 días, 17:23</t>
         </is>
       </c>
     </row>
@@ -2455,11 +2455,11 @@
         <v>46112.63163194444</v>
       </c>
       <c r="G57" s="2" t="n">
-        <v>0.07643933295138888</v>
+        <v>0.7247239698032407</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>0 días, 01:50</t>
+          <t>0 días, 17:23</t>
         </is>
       </c>
     </row>
@@ -2491,11 +2491,11 @@
         <v>46112.63296296296</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>0.07510831443287037</v>
+        <v>0.7233929512847223</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>0 días, 01:48</t>
+          <t>0 días, 17:21</t>
         </is>
       </c>
     </row>
@@ -2527,11 +2527,11 @@
         <v>46112.63335648148</v>
       </c>
       <c r="G59" s="2" t="n">
-        <v>0.07471479591435184</v>
+        <v>0.7229994327662037</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>0 días, 01:47</t>
+          <t>0 días, 17:21</t>
         </is>
       </c>
     </row>

</xml_diff>